<commit_message>
Update cost workbook and item catalog inputs
Publish the latest English cost workbook, revised Pathfinder BOM, Material Pricing model, and reduced item-catalog XLSX/CSV inputs for the weight, dimensions, and NCM enrichment work.
</commit_message>
<xml_diff>
--- a/Pathfinder BOM.xlsx
+++ b/Pathfinder BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matheus.deoliveira\Documents\Proposal\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wabtec-my.sharepoint.com/personal/matheus_deoliveira_wabtec_com/Documents/Documents/wabtec/Advanced Technology/MRS/Proposal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FF3E4B-1599-4F99-8314-E977944611AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{29FF3E4B-1599-4F99-8314-E977944611AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0930A517-3BCD-4345-BD93-F16EFD50EA3D}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{3D31F91C-8345-477C-B634-69BA23E15693}"/>
+    <workbookView xWindow="7335" yWindow="3795" windowWidth="21465" windowHeight="11025" xr2:uid="{3D31F91C-8345-477C-B634-69BA23E15693}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Z$282</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -8590,7 +8591,7 @@
       <c r="Y118" s="2"/>
       <c r="Z118" s="2"/>
     </row>
-    <row r="119" spans="1:26" ht="30" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>13</v>
       </c>
@@ -11117,7 +11118,7 @@
       <c r="Y178" s="2"/>
       <c r="Z178" s="2"/>
     </row>
-    <row r="179" spans="1:26" ht="30" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>13</v>
       </c>
@@ -14910,7 +14911,11 @@
       <c r="Z282" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z282" xr:uid="{05F2BE3D-6BE4-412D-94D1-37A54DF02A1D}"/>
+  <autoFilter ref="A1:Z282" xr:uid="{05F2BE3D-6BE4-412D-94D1-37A54DF02A1D}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Z282">
+      <sortCondition descending="1" ref="P1:P282"/>
+    </sortState>
+  </autoFilter>
   <conditionalFormatting sqref="D57:D65">
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>

</xml_diff>